<commit_message>
implement heigh sensor basics and EEPROM
</commit_message>
<xml_diff>
--- a/PGN 5.7_planter.xlsx
+++ b/PGN 5.7_planter.xlsx
@@ -11,7 +11,7 @@
     <sheet name="PGN" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">PGN!$A$1:$Q$114</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">PGN!$A$1:$Q$124</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="369">
   <si>
     <t xml:space="preserve">PGN Name</t>
   </si>
@@ -739,15 +739,9 @@
     <t xml:space="preserve">old, not used</t>
   </si>
   <si>
-    <t xml:space="preserve">IP = 192.168.1.192</t>
-  </si>
-  <si>
     <t xml:space="preserve">Array Doubles</t>
   </si>
   <si>
-    <t xml:space="preserve">Hello = 9998?</t>
-  </si>
-  <si>
     <t xml:space="preserve">Row Status</t>
   </si>
   <si>
@@ -775,9 +769,6 @@
     <t xml:space="preserve">On is 0, off is 1, for compatibility</t>
   </si>
   <si>
-    <t xml:space="preserve">Port = 9998</t>
-  </si>
-  <si>
     <t xml:space="preserve">Summary</t>
   </si>
   <si>
@@ -866,6 +857,162 @@
   </si>
   <si>
     <t xml:space="preserve">Off Group 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planter Comms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Height</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw Hi/Lo 0-4095(0-12v)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Height 0-255</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Off threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Height config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zero Hi/Lo 1-4095 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOP Hi/Lo 1-4095 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On threshold 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Off threshold 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vacuum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inWC1X10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inWC2X10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vacuum config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zero1 Hi/Lo 1-4095 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zero2 Hi/Lo 1-4095 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act inWCX10 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downpressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sen1 (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sen2 (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sen3 (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">airDwPres PSI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status bits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status bit :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 israising</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 islowering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 pressSwt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 isAuto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downpressure config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act weight(kg), 0 = no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">set0,1=true,bit = sensNbr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act PressPSI 0= no data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 raisePres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 lowerPres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fertilizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(signed)weight (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act pos 1-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act pos 9-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set pos 1-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set pos 9-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fertilizer config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ForceOn 1-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ForceOn 9-16</t>
   </si>
   <si>
     <t xml:space="preserve">Hello Sent To Module</t>
@@ -1348,7 +1495,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="117">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1723,6 +1870,62 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2012,7 +2215,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:AP113"/>
+  <dimension ref="A1:AP123"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.42"/>
@@ -2026,7 +2229,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="9" width="14.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="10" style="10" width="14.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="10" width="12.71"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="18" min="18" style="10" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="10" width="10.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="10" width="6.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="20" style="10" width="5.71"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="41" style="1" width="9.14"/>
@@ -4323,11 +4526,9 @@
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="69"/>
-      <c r="B76" s="49" t="s">
+      <c r="B76" s="49"/>
+      <c r="C76" s="79" t="s">
         <v>238</v>
-      </c>
-      <c r="C76" s="79" t="s">
-        <v>239</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>102</v>
@@ -4380,11 +4581,9 @@
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="69"/>
-      <c r="B77" s="49" t="s">
-        <v>240</v>
-      </c>
+      <c r="B77" s="49"/>
       <c r="C77" s="83" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>102</v>
@@ -4400,32 +4599,32 @@
         <v>8</v>
       </c>
       <c r="I77" s="85" t="s">
+        <v>240</v>
+      </c>
+      <c r="J77" s="85" t="s">
+        <v>241</v>
+      </c>
+      <c r="K77" s="85" t="s">
         <v>242</v>
       </c>
-      <c r="J77" s="85" t="s">
+      <c r="L77" s="85" t="s">
         <v>243</v>
       </c>
-      <c r="K77" s="85" t="s">
+      <c r="M77" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="L77" s="85" t="s">
+      <c r="N77" s="85" t="s">
         <v>245</v>
       </c>
-      <c r="M77" s="85" t="s">
+      <c r="O77" s="85" t="s">
         <v>246</v>
-      </c>
-      <c r="N77" s="85" t="s">
-        <v>247</v>
-      </c>
-      <c r="O77" s="85" t="s">
-        <v>248</v>
       </c>
       <c r="P77" s="86"/>
       <c r="Q77" s="84" t="s">
         <v>25</v>
       </c>
       <c r="R77" s="85" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="S77" s="85"/>
       <c r="T77" s="85"/>
@@ -4435,11 +4634,9 @@
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="69"/>
-      <c r="B78" s="49" t="s">
-        <v>250</v>
-      </c>
+      <c r="B78" s="49"/>
       <c r="C78" s="76" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>102</v>
@@ -4455,19 +4652,19 @@
         <v>8</v>
       </c>
       <c r="I78" s="87" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J78" s="87"/>
       <c r="K78" s="8" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="L78" s="8"/>
       <c r="M78" s="8" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="N78" s="8"/>
       <c r="O78" s="8" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="P78" s="8"/>
       <c r="Q78" s="78" t="s">
@@ -4477,14 +4674,14 @@
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="69"/>
       <c r="C79" s="76" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>102</v>
       </c>
       <c r="E79" s="77"/>
       <c r="F79" s="6" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="G79" s="7" t="n">
         <v>228</v>
@@ -4520,7 +4717,7 @@
         <v>25</v>
       </c>
       <c r="R79" s="8" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="S79" s="8"/>
       <c r="T79" s="8"/>
@@ -4530,14 +4727,14 @@
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="69"/>
       <c r="C80" s="76" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>102</v>
       </c>
       <c r="E80" s="77"/>
       <c r="F80" s="6" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="G80" s="7" t="n">
         <v>227</v>
@@ -4576,14 +4773,14 @@
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="69"/>
       <c r="C81" s="76" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>102</v>
       </c>
       <c r="E81" s="77"/>
       <c r="F81" s="6" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="G81" s="7" t="n">
         <v>226</v>
@@ -4622,14 +4819,14 @@
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="69"/>
       <c r="C82" s="76" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>102</v>
       </c>
       <c r="E82" s="77"/>
       <c r="F82" s="6" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="G82" s="7" t="n">
         <v>225</v>
@@ -4669,14 +4866,14 @@
       <c r="A83" s="88"/>
       <c r="B83" s="51"/>
       <c r="C83" s="89" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D83" s="53" t="s">
         <v>102</v>
       </c>
       <c r="E83" s="90"/>
       <c r="F83" s="55" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="G83" s="56" t="n">
         <v>224</v>
@@ -4685,24 +4882,24 @@
         <v>8</v>
       </c>
       <c r="I83" s="92" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="J83" s="92" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="K83" s="92" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="L83" s="92"/>
       <c r="M83" s="57" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="N83" s="57"/>
       <c r="O83" s="92" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="P83" s="57" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="Q83" s="91" t="s">
         <v>25</v>
@@ -4752,7 +4949,7 @@
     <row r="85" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="49"/>
       <c r="C85" s="3" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D85" s="4" t="n">
         <v>77</v>
@@ -4761,35 +4958,35 @@
         <v>119</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G85" s="7" t="n">
         <v>234</v>
       </c>
       <c r="H85" s="8"/>
       <c r="I85" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="J85" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="K85" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="L85" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="M85" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="J85" s="8" t="s">
+      <c r="N85" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="K85" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="L85" s="8" t="s">
+      <c r="O85" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="M85" s="8" t="s">
+      <c r="P85" s="8" t="s">
         <v>277</v>
-      </c>
-      <c r="N85" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="O85" s="8" t="s">
-        <v>279</v>
-      </c>
-      <c r="P85" s="8" t="s">
-        <v>280</v>
       </c>
       <c r="Q85" s="8" t="s">
         <v>25</v>
@@ -4900,82 +5097,86 @@
       <c r="AM87" s="57"/>
       <c r="AN87" s="57"/>
     </row>
-    <row r="88" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B88" s="49"/>
-      <c r="C88" s="3"/>
-      <c r="D88" s="4"/>
-      <c r="E88" s="5"/>
-      <c r="F88" s="6"/>
-      <c r="G88" s="7"/>
-      <c r="H88" s="8"/>
-      <c r="I88" s="9"/>
-      <c r="J88" s="8"/>
-      <c r="K88" s="8"/>
-      <c r="L88" s="8"/>
-      <c r="M88" s="8"/>
-      <c r="N88" s="8"/>
-      <c r="O88" s="8"/>
-      <c r="P88" s="8"/>
-      <c r="Q88" s="8"/>
-      <c r="R88" s="8"/>
-      <c r="S88" s="8"/>
-      <c r="T88" s="8"/>
-      <c r="U88" s="8"/>
-      <c r="V88" s="8"/>
-      <c r="W88" s="8"/>
-      <c r="X88" s="8"/>
-      <c r="Y88" s="8"/>
-      <c r="Z88" s="8"/>
-      <c r="AA88" s="8"/>
-      <c r="AB88" s="8"/>
-      <c r="AC88" s="8"/>
-      <c r="AD88" s="8"/>
-      <c r="AE88" s="8"/>
-      <c r="AF88" s="8"/>
-      <c r="AG88" s="8"/>
-      <c r="AH88" s="8"/>
-      <c r="AI88" s="8"/>
-      <c r="AJ88" s="8"/>
-      <c r="AK88" s="8"/>
-      <c r="AL88" s="8"/>
-      <c r="AM88" s="8"/>
-      <c r="AN88" s="8"/>
+    <row r="88" s="50" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B88" s="94" t="s">
+        <v>278</v>
+      </c>
+      <c r="C88" s="52"/>
+      <c r="D88" s="53"/>
+      <c r="E88" s="54"/>
+      <c r="F88" s="55"/>
+      <c r="G88" s="56"/>
+      <c r="H88" s="57"/>
+      <c r="I88" s="58"/>
+      <c r="J88" s="57"/>
+      <c r="K88" s="57"/>
+      <c r="L88" s="57"/>
+      <c r="M88" s="57"/>
+      <c r="N88" s="57"/>
+      <c r="O88" s="57"/>
+      <c r="P88" s="57"/>
+      <c r="Q88" s="57"/>
+      <c r="R88" s="57"/>
+      <c r="S88" s="57"/>
+      <c r="T88" s="57"/>
+      <c r="U88" s="57"/>
+      <c r="V88" s="57"/>
+      <c r="W88" s="57"/>
+      <c r="X88" s="57"/>
+      <c r="Y88" s="57"/>
+      <c r="Z88" s="57"/>
+      <c r="AA88" s="57"/>
+      <c r="AB88" s="57"/>
+      <c r="AC88" s="57"/>
+      <c r="AD88" s="57"/>
+      <c r="AE88" s="57"/>
+      <c r="AF88" s="57"/>
+      <c r="AG88" s="57"/>
+      <c r="AH88" s="57"/>
+      <c r="AI88" s="57"/>
+      <c r="AJ88" s="57"/>
+      <c r="AK88" s="57"/>
+      <c r="AL88" s="57"/>
+      <c r="AM88" s="57"/>
+      <c r="AN88" s="57"/>
     </row>
     <row r="89" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B89" s="49" t="s">
+      <c r="B89" s="49"/>
+      <c r="C89" s="95" t="s">
+        <v>279</v>
+      </c>
+      <c r="D89" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E89" s="97"/>
+      <c r="F89" s="98" t="s">
+        <v>280</v>
+      </c>
+      <c r="G89" s="99" t="n">
+        <v>160</v>
+      </c>
+      <c r="H89" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I89" s="100" t="s">
         <v>281</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="J89" s="100"/>
+      <c r="K89" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="D89" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E89" s="5"/>
-      <c r="F89" s="6"/>
-      <c r="G89" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="H89" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="I89" s="9" t="s">
+      <c r="L89" s="101"/>
+      <c r="M89" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="J89" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K89" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L89" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="M89" s="8"/>
-      <c r="N89" s="8"/>
+      <c r="N89" s="8" t="s">
+        <v>284</v>
+      </c>
       <c r="O89" s="8"/>
       <c r="P89" s="8"/>
-      <c r="Q89" s="8"/>
+      <c r="Q89" s="87" t="s">
+        <v>25</v>
+      </c>
       <c r="R89" s="8"/>
       <c r="S89" s="8"/>
       <c r="T89" s="8"/>
@@ -5000,23 +5201,43 @@
       <c r="AM89" s="8"/>
       <c r="AN89" s="8"/>
     </row>
-    <row r="90" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B90" s="94"/>
-      <c r="C90" s="3"/>
-      <c r="D90" s="4"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="6"/>
-      <c r="G90" s="7"/>
-      <c r="H90" s="8"/>
-      <c r="I90" s="9"/>
-      <c r="J90" s="8"/>
-      <c r="K90" s="8"/>
-      <c r="L90" s="8"/>
-      <c r="M90" s="8"/>
-      <c r="N90" s="8"/>
+    <row r="90" s="59" customFormat="true" ht="29.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B90" s="49"/>
+      <c r="C90" s="95" t="s">
+        <v>285</v>
+      </c>
+      <c r="D90" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E90" s="97"/>
+      <c r="F90" s="98" t="s">
+        <v>286</v>
+      </c>
+      <c r="G90" s="99" t="n">
+        <v>161</v>
+      </c>
+      <c r="H90" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I90" s="100" t="s">
+        <v>287</v>
+      </c>
+      <c r="J90" s="100"/>
+      <c r="K90" s="100" t="s">
+        <v>288</v>
+      </c>
+      <c r="L90" s="100"/>
+      <c r="M90" s="102" t="s">
+        <v>289</v>
+      </c>
+      <c r="N90" s="102" t="s">
+        <v>290</v>
+      </c>
       <c r="O90" s="8"/>
       <c r="P90" s="8"/>
-      <c r="Q90" s="8"/>
+      <c r="Q90" s="87" t="s">
+        <v>25</v>
+      </c>
       <c r="R90" s="8"/>
       <c r="S90" s="8"/>
       <c r="T90" s="8"/>
@@ -5042,44 +5263,42 @@
       <c r="AN90" s="8"/>
     </row>
     <row r="91" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B91" s="49" t="s">
-        <v>284</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D91" s="4" t="n">
-        <v>126</v>
-      </c>
-      <c r="E91" s="5"/>
-      <c r="F91" s="6"/>
-      <c r="G91" s="7" t="n">
-        <v>126</v>
+      <c r="B91" s="49"/>
+      <c r="C91" s="95" t="s">
+        <v>291</v>
+      </c>
+      <c r="D91" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E91" s="97"/>
+      <c r="F91" s="98" t="s">
+        <v>292</v>
+      </c>
+      <c r="G91" s="99" t="n">
+        <v>162</v>
       </c>
       <c r="H91" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="I91" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="J91" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="K91" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="L91" s="8" t="s">
-        <v>289</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="I91" s="100" t="s">
+        <v>281</v>
+      </c>
+      <c r="J91" s="100"/>
+      <c r="K91" s="100" t="s">
+        <v>281</v>
+      </c>
+      <c r="L91" s="100"/>
       <c r="M91" s="8" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="N91" s="8" t="s">
-        <v>25</v>
+        <v>294</v>
       </c>
       <c r="O91" s="8"/>
       <c r="P91" s="8"/>
-      <c r="Q91" s="8"/>
+      <c r="Q91" s="87" t="s">
+        <v>25</v>
+      </c>
       <c r="R91" s="8"/>
       <c r="S91" s="8"/>
       <c r="T91" s="8"/>
@@ -5104,43 +5323,43 @@
       <c r="AM91" s="8"/>
       <c r="AN91" s="8"/>
     </row>
-    <row r="92" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B92" s="94"/>
-      <c r="C92" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="D92" s="4" t="n">
-        <v>123</v>
-      </c>
-      <c r="E92" s="5"/>
-      <c r="F92" s="6"/>
-      <c r="G92" s="7" t="n">
-        <v>123</v>
+    <row r="92" s="59" customFormat="true" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B92" s="49"/>
+      <c r="C92" s="95" t="s">
+        <v>295</v>
+      </c>
+      <c r="D92" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E92" s="97"/>
+      <c r="F92" s="98" t="s">
+        <v>296</v>
+      </c>
+      <c r="G92" s="99" t="n">
+        <v>163</v>
       </c>
       <c r="H92" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="I92" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="J92" s="8" t="s">
-        <v>293</v>
-      </c>
-      <c r="K92" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="L92" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="M92" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="N92" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="I92" s="100" t="s">
+        <v>297</v>
+      </c>
+      <c r="J92" s="100"/>
+      <c r="K92" s="100" t="s">
+        <v>298</v>
+      </c>
+      <c r="L92" s="100"/>
+      <c r="M92" s="103" t="s">
+        <v>299</v>
+      </c>
+      <c r="N92" s="103" t="s">
+        <v>299</v>
+      </c>
+      <c r="O92" s="100"/>
+      <c r="P92" s="8"/>
+      <c r="Q92" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="O92" s="8"/>
-      <c r="P92" s="8"/>
-      <c r="Q92" s="8"/>
       <c r="R92" s="8"/>
       <c r="S92" s="8"/>
       <c r="T92" s="8"/>
@@ -5166,50 +5385,64 @@
       <c r="AN92" s="8"/>
     </row>
     <row r="93" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B93" s="94"/>
-      <c r="C93" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="D93" s="4" t="n">
-        <v>121</v>
-      </c>
-      <c r="E93" s="5"/>
-      <c r="F93" s="6"/>
-      <c r="G93" s="7" t="n">
-        <v>121</v>
+      <c r="B93" s="49"/>
+      <c r="C93" s="95" t="s">
+        <v>300</v>
+      </c>
+      <c r="D93" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E93" s="97"/>
+      <c r="F93" s="98" t="s">
+        <v>301</v>
+      </c>
+      <c r="G93" s="99" t="n">
+        <v>164</v>
       </c>
       <c r="H93" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I93" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="J93" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="K93" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="L93" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="M93" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="N93" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="J93" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="K93" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="L93" s="101"/>
+      <c r="M93" s="100" t="s">
+        <v>281</v>
+      </c>
+      <c r="N93" s="100"/>
+      <c r="O93" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="P93" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="Q93" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="O93" s="8"/>
-      <c r="P93" s="8"/>
-      <c r="Q93" s="8"/>
-      <c r="R93" s="8"/>
-      <c r="S93" s="8"/>
-      <c r="T93" s="8"/>
-      <c r="U93" s="8"/>
+      <c r="R93" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="S93" s="87" t="s">
+        <v>308</v>
+      </c>
+      <c r="T93" s="87"/>
+      <c r="U93" s="8" t="s">
+        <v>309</v>
+      </c>
       <c r="V93" s="8"/>
-      <c r="W93" s="8"/>
+      <c r="W93" s="8" t="s">
+        <v>310</v>
+      </c>
       <c r="X93" s="8"/>
-      <c r="Y93" s="8"/>
+      <c r="Y93" s="8" t="s">
+        <v>311</v>
+      </c>
       <c r="Z93" s="8"/>
       <c r="AA93" s="8"/>
       <c r="AB93" s="8"/>
@@ -5226,52 +5459,66 @@
       <c r="AM93" s="8"/>
       <c r="AN93" s="8"/>
     </row>
-    <row r="94" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B94" s="94"/>
-      <c r="C94" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="D94" s="4" t="n">
-        <v>120</v>
-      </c>
-      <c r="E94" s="5"/>
-      <c r="F94" s="6"/>
-      <c r="G94" s="7" t="n">
-        <v>120</v>
+    <row r="94" s="59" customFormat="true" ht="30.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B94" s="49"/>
+      <c r="C94" s="104" t="s">
+        <v>312</v>
+      </c>
+      <c r="D94" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E94" s="97"/>
+      <c r="F94" s="98" t="s">
+        <v>313</v>
+      </c>
+      <c r="G94" s="99" t="n">
+        <v>165</v>
       </c>
       <c r="H94" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="I94" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="J94" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="K94" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="L94" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="M94" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="N94" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="I94" s="105" t="s">
+        <v>314</v>
+      </c>
+      <c r="J94" s="105" t="s">
+        <v>314</v>
+      </c>
+      <c r="K94" s="105" t="s">
+        <v>314</v>
+      </c>
+      <c r="L94" s="106" t="s">
+        <v>315</v>
+      </c>
+      <c r="M94" s="107" t="s">
+        <v>287</v>
+      </c>
+      <c r="N94" s="107"/>
+      <c r="O94" s="103" t="s">
+        <v>316</v>
+      </c>
+      <c r="P94" s="87" t="s">
+        <v>306</v>
+      </c>
+      <c r="Q94" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="O94" s="8"/>
-      <c r="P94" s="8"/>
-      <c r="Q94" s="8"/>
-      <c r="R94" s="8"/>
-      <c r="S94" s="8"/>
-      <c r="T94" s="8"/>
-      <c r="U94" s="8"/>
-      <c r="V94" s="8"/>
-      <c r="W94" s="8"/>
-      <c r="X94" s="8"/>
-      <c r="Y94" s="8"/>
-      <c r="Z94" s="8"/>
+      <c r="R94" s="87" t="s">
+        <v>307</v>
+      </c>
+      <c r="S94" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="T94" s="87"/>
+      <c r="U94" s="87" t="s">
+        <v>318</v>
+      </c>
+      <c r="V94" s="87"/>
+      <c r="W94" s="87"/>
+      <c r="X94" s="87"/>
+      <c r="Y94" s="87" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z94" s="87"/>
       <c r="AA94" s="8"/>
       <c r="AB94" s="8"/>
       <c r="AC94" s="8"/>
@@ -5289,21 +5536,43 @@
     </row>
     <row r="95" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="49"/>
-      <c r="C95" s="3"/>
-      <c r="D95" s="4"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="6"/>
-      <c r="G95" s="7"/>
-      <c r="H95" s="8"/>
-      <c r="I95" s="9"/>
-      <c r="J95" s="8"/>
-      <c r="K95" s="8"/>
-      <c r="L95" s="8"/>
-      <c r="M95" s="8"/>
-      <c r="N95" s="8"/>
+      <c r="C95" s="95" t="s">
+        <v>319</v>
+      </c>
+      <c r="D95" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E95" s="97"/>
+      <c r="F95" s="98" t="s">
+        <v>320</v>
+      </c>
+      <c r="G95" s="99" t="n">
+        <v>166</v>
+      </c>
+      <c r="H95" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I95" s="100" t="s">
+        <v>321</v>
+      </c>
+      <c r="J95" s="100"/>
+      <c r="K95" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="L95" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="M95" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="N95" s="8" t="s">
+        <v>325</v>
+      </c>
       <c r="O95" s="8"/>
       <c r="P95" s="8"/>
-      <c r="Q95" s="8"/>
+      <c r="Q95" s="87" t="s">
+        <v>25</v>
+      </c>
       <c r="R95" s="8"/>
       <c r="S95" s="8"/>
       <c r="T95" s="8"/>
@@ -5329,44 +5598,38 @@
       <c r="AN95" s="8"/>
     </row>
     <row r="96" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B96" s="49" t="s">
-        <v>296</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E96" s="5"/>
-      <c r="F96" s="6"/>
-      <c r="G96" s="7" t="n">
-        <v>201</v>
+      <c r="B96" s="49"/>
+      <c r="C96" s="95" t="s">
+        <v>326</v>
+      </c>
+      <c r="D96" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="E96" s="97"/>
+      <c r="F96" s="98" t="s">
+        <v>327</v>
+      </c>
+      <c r="G96" s="99" t="n">
+        <v>167</v>
       </c>
       <c r="H96" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="I96" s="9" t="n">
-        <v>201</v>
-      </c>
-      <c r="J96" s="8" t="n">
-        <v>201</v>
-      </c>
-      <c r="K96" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="L96" s="8" t="s">
-        <v>299</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="I96" s="9"/>
+      <c r="J96" s="8"/>
+      <c r="K96" s="101"/>
+      <c r="L96" s="101"/>
       <c r="M96" s="8" t="s">
-        <v>300</v>
+        <v>328</v>
       </c>
       <c r="N96" s="8" t="s">
-        <v>25</v>
+        <v>329</v>
       </c>
       <c r="O96" s="8"/>
       <c r="P96" s="8"/>
-      <c r="Q96" s="8"/>
+      <c r="Q96" s="87" t="s">
+        <v>25</v>
+      </c>
       <c r="R96" s="8"/>
       <c r="S96" s="8"/>
       <c r="T96" s="8"/>
@@ -5433,35 +5696,17 @@
       <c r="AN97" s="8"/>
     </row>
     <row r="98" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B98" s="49" t="s">
-        <v>296</v>
-      </c>
-      <c r="C98" s="95" t="s">
-        <v>301</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="B98" s="49"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="4"/>
       <c r="E98" s="5"/>
       <c r="F98" s="6"/>
-      <c r="G98" s="7" t="n">
-        <v>202</v>
-      </c>
-      <c r="H98" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="I98" s="9" t="n">
-        <v>202</v>
-      </c>
-      <c r="J98" s="8" t="n">
-        <v>202</v>
-      </c>
-      <c r="K98" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L98" s="8" t="s">
-        <v>25</v>
-      </c>
+      <c r="G98" s="7"/>
+      <c r="H98" s="8"/>
+      <c r="I98" s="9"/>
+      <c r="J98" s="8"/>
+      <c r="K98" s="8"/>
+      <c r="L98" s="8"/>
       <c r="M98" s="8"/>
       <c r="N98" s="8"/>
       <c r="O98" s="8"/>
@@ -5492,17 +5737,35 @@
       <c r="AN98" s="8"/>
     </row>
     <row r="99" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B99" s="49"/>
-      <c r="C99" s="95"/>
-      <c r="D99" s="4"/>
+      <c r="B99" s="49" t="s">
+        <v>330</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="E99" s="5"/>
       <c r="F99" s="6"/>
-      <c r="G99" s="7"/>
-      <c r="H99" s="8"/>
-      <c r="I99" s="9"/>
-      <c r="J99" s="8"/>
-      <c r="K99" s="8"/>
-      <c r="L99" s="8"/>
+      <c r="G99" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I99" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="J99" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="M99" s="8"/>
       <c r="N99" s="8"/>
       <c r="O99" s="8"/>
@@ -5533,47 +5796,21 @@
       <c r="AN99" s="8"/>
     </row>
     <row r="100" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B100" s="49" t="s">
-        <v>302</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="D100" s="96" t="n">
-        <v>126</v>
-      </c>
+      <c r="B100" s="108"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="4"/>
       <c r="E100" s="5"/>
       <c r="F100" s="6"/>
-      <c r="G100" s="7" t="n">
-        <v>203</v>
-      </c>
-      <c r="H100" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="I100" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="J100" s="8" t="s">
-        <v>305</v>
-      </c>
-      <c r="K100" s="8" t="s">
-        <v>306</v>
-      </c>
-      <c r="L100" s="8" t="n">
-        <v>126</v>
-      </c>
-      <c r="M100" s="8" t="s">
-        <v>307</v>
-      </c>
-      <c r="N100" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="O100" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="P100" s="8" t="s">
-        <v>25</v>
-      </c>
+      <c r="G100" s="7"/>
+      <c r="H100" s="8"/>
+      <c r="I100" s="9"/>
+      <c r="J100" s="8"/>
+      <c r="K100" s="8"/>
+      <c r="L100" s="8"/>
+      <c r="M100" s="8"/>
+      <c r="N100" s="8"/>
+      <c r="O100" s="8"/>
+      <c r="P100" s="8"/>
       <c r="Q100" s="8"/>
       <c r="R100" s="8"/>
       <c r="S100" s="8"/>
@@ -5600,45 +5837,43 @@
       <c r="AN100" s="8"/>
     </row>
     <row r="101" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B101" s="49"/>
+      <c r="B101" s="49" t="s">
+        <v>333</v>
+      </c>
       <c r="C101" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="D101" s="96" t="n">
-        <v>123</v>
+        <v>334</v>
+      </c>
+      <c r="D101" s="4" t="n">
+        <v>126</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="6"/>
       <c r="G101" s="7" t="n">
-        <v>203</v>
+        <v>126</v>
       </c>
       <c r="H101" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I101" s="9" t="s">
-        <v>304</v>
+        <v>335</v>
       </c>
       <c r="J101" s="8" t="s">
-        <v>305</v>
+        <v>336</v>
       </c>
       <c r="K101" s="8" t="s">
-        <v>306</v>
-      </c>
-      <c r="L101" s="8" t="n">
-        <v>123</v>
+        <v>337</v>
+      </c>
+      <c r="L101" s="8" t="s">
+        <v>338</v>
       </c>
       <c r="M101" s="8" t="s">
-        <v>307</v>
+        <v>339</v>
       </c>
       <c r="N101" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="O101" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="P101" s="8" t="s">
         <v>25</v>
       </c>
+      <c r="O101" s="8"/>
+      <c r="P101" s="8"/>
       <c r="Q101" s="8"/>
       <c r="R101" s="8"/>
       <c r="S101" s="8"/>
@@ -5665,45 +5900,41 @@
       <c r="AN101" s="8"/>
     </row>
     <row r="102" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B102" s="49"/>
+      <c r="B102" s="108"/>
       <c r="C102" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="D102" s="96" t="n">
-        <v>121</v>
+        <v>340</v>
+      </c>
+      <c r="D102" s="4" t="n">
+        <v>123</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="6"/>
       <c r="G102" s="7" t="n">
-        <v>203</v>
+        <v>123</v>
       </c>
       <c r="H102" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I102" s="9" t="s">
-        <v>304</v>
+        <v>341</v>
       </c>
       <c r="J102" s="8" t="s">
-        <v>305</v>
+        <v>342</v>
       </c>
       <c r="K102" s="8" t="s">
-        <v>306</v>
-      </c>
-      <c r="L102" s="8" t="n">
-        <v>121</v>
+        <v>57</v>
+      </c>
+      <c r="L102" s="8" t="s">
+        <v>57</v>
       </c>
       <c r="M102" s="8" t="s">
-        <v>307</v>
+        <v>57</v>
       </c>
       <c r="N102" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="O102" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="P102" s="8" t="s">
         <v>25</v>
       </c>
+      <c r="O102" s="8"/>
+      <c r="P102" s="8"/>
       <c r="Q102" s="8"/>
       <c r="R102" s="8"/>
       <c r="S102" s="8"/>
@@ -5730,45 +5961,41 @@
       <c r="AN102" s="8"/>
     </row>
     <row r="103" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B103" s="49"/>
+      <c r="B103" s="108"/>
       <c r="C103" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="D103" s="96" t="n">
-        <v>120</v>
+        <v>343</v>
+      </c>
+      <c r="D103" s="4" t="n">
+        <v>121</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="6"/>
       <c r="G103" s="7" t="n">
-        <v>203</v>
+        <v>121</v>
       </c>
       <c r="H103" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I103" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="J103" s="8" t="s">
-        <v>305</v>
-      </c>
-      <c r="K103" s="8" t="s">
-        <v>306</v>
-      </c>
-      <c r="L103" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="M103" s="8" t="s">
-        <v>307</v>
+        <v>57</v>
+      </c>
+      <c r="J103" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K103" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="L103" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="M103" s="9" t="s">
+        <v>57</v>
       </c>
       <c r="N103" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="O103" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="P103" s="8" t="s">
         <v>25</v>
       </c>
+      <c r="O103" s="8"/>
+      <c r="P103" s="8"/>
       <c r="Q103" s="8"/>
       <c r="R103" s="8"/>
       <c r="S103" s="8"/>
@@ -5795,19 +6022,39 @@
       <c r="AN103" s="8"/>
     </row>
     <row r="104" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B104" s="49"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="96"/>
+      <c r="B104" s="108"/>
+      <c r="C104" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="D104" s="4" t="n">
+        <v>120</v>
+      </c>
       <c r="E104" s="5"/>
       <c r="F104" s="6"/>
-      <c r="G104" s="7"/>
-      <c r="H104" s="8"/>
-      <c r="I104" s="9"/>
-      <c r="J104" s="8"/>
-      <c r="K104" s="8"/>
-      <c r="L104" s="8"/>
-      <c r="M104" s="8"/>
-      <c r="N104" s="8"/>
+      <c r="G104" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H104" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I104" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J104" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K104" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="L104" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="M104" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="N104" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="O104" s="8"/>
       <c r="P104" s="8"/>
       <c r="Q104" s="8"/>
@@ -5835,95 +6082,643 @@
       <c r="AM104" s="8"/>
       <c r="AN104" s="8"/>
     </row>
-    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C106" s="97" t="s">
-        <v>313</v>
-      </c>
-      <c r="D106" s="98" t="s">
-        <v>314</v>
-      </c>
-      <c r="E106" s="99"/>
-      <c r="F106" s="100" t="s">
-        <v>315</v>
-      </c>
-      <c r="G106" s="56"/>
-    </row>
-    <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B107" s="101" t="s">
+    <row r="105" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B105" s="49"/>
+      <c r="C105" s="3"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="5"/>
+      <c r="F105" s="6"/>
+      <c r="G105" s="7"/>
+      <c r="H105" s="8"/>
+      <c r="I105" s="9"/>
+      <c r="J105" s="8"/>
+      <c r="K105" s="8"/>
+      <c r="L105" s="8"/>
+      <c r="M105" s="8"/>
+      <c r="N105" s="8"/>
+      <c r="O105" s="8"/>
+      <c r="P105" s="8"/>
+      <c r="Q105" s="8"/>
+      <c r="R105" s="8"/>
+      <c r="S105" s="8"/>
+      <c r="T105" s="8"/>
+      <c r="U105" s="8"/>
+      <c r="V105" s="8"/>
+      <c r="W105" s="8"/>
+      <c r="X105" s="8"/>
+      <c r="Y105" s="8"/>
+      <c r="Z105" s="8"/>
+      <c r="AA105" s="8"/>
+      <c r="AB105" s="8"/>
+      <c r="AC105" s="8"/>
+      <c r="AD105" s="8"/>
+      <c r="AE105" s="8"/>
+      <c r="AF105" s="8"/>
+      <c r="AG105" s="8"/>
+      <c r="AH105" s="8"/>
+      <c r="AI105" s="8"/>
+      <c r="AJ105" s="8"/>
+      <c r="AK105" s="8"/>
+      <c r="AL105" s="8"/>
+      <c r="AM105" s="8"/>
+      <c r="AN105" s="8"/>
+    </row>
+    <row r="106" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B106" s="49" t="s">
+        <v>345</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E106" s="5"/>
+      <c r="F106" s="6"/>
+      <c r="G106" s="7" t="n">
+        <v>201</v>
+      </c>
+      <c r="H106" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I106" s="9" t="n">
+        <v>201</v>
+      </c>
+      <c r="J106" s="8" t="n">
+        <v>201</v>
+      </c>
+      <c r="K106" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="L106" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="M106" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="N106" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O106" s="8"/>
+      <c r="P106" s="8"/>
+      <c r="Q106" s="8"/>
+      <c r="R106" s="8"/>
+      <c r="S106" s="8"/>
+      <c r="T106" s="8"/>
+      <c r="U106" s="8"/>
+      <c r="V106" s="8"/>
+      <c r="W106" s="8"/>
+      <c r="X106" s="8"/>
+      <c r="Y106" s="8"/>
+      <c r="Z106" s="8"/>
+      <c r="AA106" s="8"/>
+      <c r="AB106" s="8"/>
+      <c r="AC106" s="8"/>
+      <c r="AD106" s="8"/>
+      <c r="AE106" s="8"/>
+      <c r="AF106" s="8"/>
+      <c r="AG106" s="8"/>
+      <c r="AH106" s="8"/>
+      <c r="AI106" s="8"/>
+      <c r="AJ106" s="8"/>
+      <c r="AK106" s="8"/>
+      <c r="AL106" s="8"/>
+      <c r="AM106" s="8"/>
+      <c r="AN106" s="8"/>
+    </row>
+    <row r="107" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B107" s="49"/>
+      <c r="C107" s="3"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="5"/>
+      <c r="F107" s="6"/>
+      <c r="G107" s="7"/>
+      <c r="H107" s="8"/>
+      <c r="I107" s="9"/>
+      <c r="J107" s="8"/>
+      <c r="K107" s="8"/>
+      <c r="L107" s="8"/>
+      <c r="M107" s="8"/>
+      <c r="N107" s="8"/>
+      <c r="O107" s="8"/>
+      <c r="P107" s="8"/>
+      <c r="Q107" s="8"/>
+      <c r="R107" s="8"/>
+      <c r="S107" s="8"/>
+      <c r="T107" s="8"/>
+      <c r="U107" s="8"/>
+      <c r="V107" s="8"/>
+      <c r="W107" s="8"/>
+      <c r="X107" s="8"/>
+      <c r="Y107" s="8"/>
+      <c r="Z107" s="8"/>
+      <c r="AA107" s="8"/>
+      <c r="AB107" s="8"/>
+      <c r="AC107" s="8"/>
+      <c r="AD107" s="8"/>
+      <c r="AE107" s="8"/>
+      <c r="AF107" s="8"/>
+      <c r="AG107" s="8"/>
+      <c r="AH107" s="8"/>
+      <c r="AI107" s="8"/>
+      <c r="AJ107" s="8"/>
+      <c r="AK107" s="8"/>
+      <c r="AL107" s="8"/>
+      <c r="AM107" s="8"/>
+      <c r="AN107" s="8"/>
+    </row>
+    <row r="108" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B108" s="49" t="s">
+        <v>345</v>
+      </c>
+      <c r="C108" s="109" t="s">
+        <v>350</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E108" s="5"/>
+      <c r="F108" s="6"/>
+      <c r="G108" s="7" t="n">
+        <v>202</v>
+      </c>
+      <c r="H108" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I108" s="9" t="n">
+        <v>202</v>
+      </c>
+      <c r="J108" s="8" t="n">
+        <v>202</v>
+      </c>
+      <c r="K108" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L108" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="M108" s="8"/>
+      <c r="N108" s="8"/>
+      <c r="O108" s="8"/>
+      <c r="P108" s="8"/>
+      <c r="Q108" s="8"/>
+      <c r="R108" s="8"/>
+      <c r="S108" s="8"/>
+      <c r="T108" s="8"/>
+      <c r="U108" s="8"/>
+      <c r="V108" s="8"/>
+      <c r="W108" s="8"/>
+      <c r="X108" s="8"/>
+      <c r="Y108" s="8"/>
+      <c r="Z108" s="8"/>
+      <c r="AA108" s="8"/>
+      <c r="AB108" s="8"/>
+      <c r="AC108" s="8"/>
+      <c r="AD108" s="8"/>
+      <c r="AE108" s="8"/>
+      <c r="AF108" s="8"/>
+      <c r="AG108" s="8"/>
+      <c r="AH108" s="8"/>
+      <c r="AI108" s="8"/>
+      <c r="AJ108" s="8"/>
+      <c r="AK108" s="8"/>
+      <c r="AL108" s="8"/>
+      <c r="AM108" s="8"/>
+      <c r="AN108" s="8"/>
+    </row>
+    <row r="109" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B109" s="49"/>
+      <c r="C109" s="109"/>
+      <c r="D109" s="4"/>
+      <c r="E109" s="5"/>
+      <c r="F109" s="6"/>
+      <c r="G109" s="7"/>
+      <c r="H109" s="8"/>
+      <c r="I109" s="9"/>
+      <c r="J109" s="8"/>
+      <c r="K109" s="8"/>
+      <c r="L109" s="8"/>
+      <c r="M109" s="8"/>
+      <c r="N109" s="8"/>
+      <c r="O109" s="8"/>
+      <c r="P109" s="8"/>
+      <c r="Q109" s="8"/>
+      <c r="R109" s="8"/>
+      <c r="S109" s="8"/>
+      <c r="T109" s="8"/>
+      <c r="U109" s="8"/>
+      <c r="V109" s="8"/>
+      <c r="W109" s="8"/>
+      <c r="X109" s="8"/>
+      <c r="Y109" s="8"/>
+      <c r="Z109" s="8"/>
+      <c r="AA109" s="8"/>
+      <c r="AB109" s="8"/>
+      <c r="AC109" s="8"/>
+      <c r="AD109" s="8"/>
+      <c r="AE109" s="8"/>
+      <c r="AF109" s="8"/>
+      <c r="AG109" s="8"/>
+      <c r="AH109" s="8"/>
+      <c r="AI109" s="8"/>
+      <c r="AJ109" s="8"/>
+      <c r="AK109" s="8"/>
+      <c r="AL109" s="8"/>
+      <c r="AM109" s="8"/>
+      <c r="AN109" s="8"/>
+    </row>
+    <row r="110" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B110" s="49" t="s">
+        <v>351</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="D110" s="110" t="n">
+        <v>126</v>
+      </c>
+      <c r="E110" s="5"/>
+      <c r="F110" s="6"/>
+      <c r="G110" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="H110" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I110" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="J110" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="K110" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="L110" s="8" t="n">
+        <v>126</v>
+      </c>
+      <c r="M110" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="N110" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="O110" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="P110" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q110" s="8"/>
+      <c r="R110" s="8"/>
+      <c r="S110" s="8"/>
+      <c r="T110" s="8"/>
+      <c r="U110" s="8"/>
+      <c r="V110" s="8"/>
+      <c r="W110" s="8"/>
+      <c r="X110" s="8"/>
+      <c r="Y110" s="8"/>
+      <c r="Z110" s="8"/>
+      <c r="AA110" s="8"/>
+      <c r="AB110" s="8"/>
+      <c r="AC110" s="8"/>
+      <c r="AD110" s="8"/>
+      <c r="AE110" s="8"/>
+      <c r="AF110" s="8"/>
+      <c r="AG110" s="8"/>
+      <c r="AH110" s="8"/>
+      <c r="AI110" s="8"/>
+      <c r="AJ110" s="8"/>
+      <c r="AK110" s="8"/>
+      <c r="AL110" s="8"/>
+      <c r="AM110" s="8"/>
+      <c r="AN110" s="8"/>
+    </row>
+    <row r="111" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B111" s="49"/>
+      <c r="C111" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="D111" s="110" t="n">
+        <v>123</v>
+      </c>
+      <c r="E111" s="5"/>
+      <c r="F111" s="6"/>
+      <c r="G111" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="H111" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I111" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="J111" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="K111" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="L111" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="M111" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="N111" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="O111" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="P111" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q111" s="8"/>
+      <c r="R111" s="8"/>
+      <c r="S111" s="8"/>
+      <c r="T111" s="8"/>
+      <c r="U111" s="8"/>
+      <c r="V111" s="8"/>
+      <c r="W111" s="8"/>
+      <c r="X111" s="8"/>
+      <c r="Y111" s="8"/>
+      <c r="Z111" s="8"/>
+      <c r="AA111" s="8"/>
+      <c r="AB111" s="8"/>
+      <c r="AC111" s="8"/>
+      <c r="AD111" s="8"/>
+      <c r="AE111" s="8"/>
+      <c r="AF111" s="8"/>
+      <c r="AG111" s="8"/>
+      <c r="AH111" s="8"/>
+      <c r="AI111" s="8"/>
+      <c r="AJ111" s="8"/>
+      <c r="AK111" s="8"/>
+      <c r="AL111" s="8"/>
+      <c r="AM111" s="8"/>
+      <c r="AN111" s="8"/>
+    </row>
+    <row r="112" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B112" s="49"/>
+      <c r="C112" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="D112" s="110" t="n">
+        <v>121</v>
+      </c>
+      <c r="E112" s="5"/>
+      <c r="F112" s="6"/>
+      <c r="G112" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="H112" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I112" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="J112" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="K112" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="L112" s="8" t="n">
+        <v>121</v>
+      </c>
+      <c r="M112" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="N112" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="O112" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="P112" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q112" s="8"/>
+      <c r="R112" s="8"/>
+      <c r="S112" s="8"/>
+      <c r="T112" s="8"/>
+      <c r="U112" s="8"/>
+      <c r="V112" s="8"/>
+      <c r="W112" s="8"/>
+      <c r="X112" s="8"/>
+      <c r="Y112" s="8"/>
+      <c r="Z112" s="8"/>
+      <c r="AA112" s="8"/>
+      <c r="AB112" s="8"/>
+      <c r="AC112" s="8"/>
+      <c r="AD112" s="8"/>
+      <c r="AE112" s="8"/>
+      <c r="AF112" s="8"/>
+      <c r="AG112" s="8"/>
+      <c r="AH112" s="8"/>
+      <c r="AI112" s="8"/>
+      <c r="AJ112" s="8"/>
+      <c r="AK112" s="8"/>
+      <c r="AL112" s="8"/>
+      <c r="AM112" s="8"/>
+      <c r="AN112" s="8"/>
+    </row>
+    <row r="113" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B113" s="49"/>
+      <c r="C113" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="D113" s="110" t="n">
+        <v>120</v>
+      </c>
+      <c r="E113" s="5"/>
+      <c r="F113" s="6"/>
+      <c r="G113" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="H113" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I113" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="J113" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="K113" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="L113" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="M113" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="N113" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="O113" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="P113" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q113" s="8"/>
+      <c r="R113" s="8"/>
+      <c r="S113" s="8"/>
+      <c r="T113" s="8"/>
+      <c r="U113" s="8"/>
+      <c r="V113" s="8"/>
+      <c r="W113" s="8"/>
+      <c r="X113" s="8"/>
+      <c r="Y113" s="8"/>
+      <c r="Z113" s="8"/>
+      <c r="AA113" s="8"/>
+      <c r="AB113" s="8"/>
+      <c r="AC113" s="8"/>
+      <c r="AD113" s="8"/>
+      <c r="AE113" s="8"/>
+      <c r="AF113" s="8"/>
+      <c r="AG113" s="8"/>
+      <c r="AH113" s="8"/>
+      <c r="AI113" s="8"/>
+      <c r="AJ113" s="8"/>
+      <c r="AK113" s="8"/>
+      <c r="AL113" s="8"/>
+      <c r="AM113" s="8"/>
+      <c r="AN113" s="8"/>
+    </row>
+    <row r="114" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B114" s="49"/>
+      <c r="C114" s="3"/>
+      <c r="D114" s="110"/>
+      <c r="E114" s="5"/>
+      <c r="F114" s="6"/>
+      <c r="G114" s="7"/>
+      <c r="H114" s="8"/>
+      <c r="I114" s="9"/>
+      <c r="J114" s="8"/>
+      <c r="K114" s="8"/>
+      <c r="L114" s="8"/>
+      <c r="M114" s="8"/>
+      <c r="N114" s="8"/>
+      <c r="O114" s="8"/>
+      <c r="P114" s="8"/>
+      <c r="Q114" s="8"/>
+      <c r="R114" s="8"/>
+      <c r="S114" s="8"/>
+      <c r="T114" s="8"/>
+      <c r="U114" s="8"/>
+      <c r="V114" s="8"/>
+      <c r="W114" s="8"/>
+      <c r="X114" s="8"/>
+      <c r="Y114" s="8"/>
+      <c r="Z114" s="8"/>
+      <c r="AA114" s="8"/>
+      <c r="AB114" s="8"/>
+      <c r="AC114" s="8"/>
+      <c r="AD114" s="8"/>
+      <c r="AE114" s="8"/>
+      <c r="AF114" s="8"/>
+      <c r="AG114" s="8"/>
+      <c r="AH114" s="8"/>
+      <c r="AI114" s="8"/>
+      <c r="AJ114" s="8"/>
+      <c r="AK114" s="8"/>
+      <c r="AL114" s="8"/>
+      <c r="AM114" s="8"/>
+      <c r="AN114" s="8"/>
+    </row>
+    <row r="116" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C116" s="111" t="s">
+        <v>362</v>
+      </c>
+      <c r="D116" s="112" t="s">
+        <v>363</v>
+      </c>
+      <c r="E116" s="113"/>
+      <c r="F116" s="114" t="s">
+        <v>364</v>
+      </c>
+      <c r="G116" s="56"/>
+    </row>
+    <row r="117" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B117" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="C107" s="102" t="s">
-        <v>316</v>
-      </c>
-      <c r="D107" s="4" t="n">
+      <c r="C117" s="116" t="s">
+        <v>365</v>
+      </c>
+      <c r="D117" s="4" t="n">
         <v>254</v>
       </c>
-      <c r="E107" s="5" t="s">
+      <c r="E117" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F107" s="6" t="n">
+      <c r="F117" s="6" t="n">
         <v>253</v>
       </c>
-      <c r="G107" s="7" t="s">
+      <c r="G117" s="7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B108" s="101"/>
-      <c r="C108" s="102"/>
-    </row>
-    <row r="109" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B109" s="101" t="s">
+    <row r="118" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B118" s="115"/>
+      <c r="C118" s="116"/>
+    </row>
+    <row r="119" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B119" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="C109" s="102" t="s">
-        <v>317</v>
-      </c>
-      <c r="D109" s="4" t="n">
+      <c r="C119" s="116" t="s">
+        <v>366</v>
+      </c>
+      <c r="D119" s="4" t="n">
         <v>239</v>
       </c>
-      <c r="E109" s="5" t="s">
+      <c r="E119" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F109" s="6" t="n">
+      <c r="F119" s="6" t="n">
         <v>237</v>
       </c>
-      <c r="G109" s="7" t="s">
+      <c r="G119" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B110" s="101"/>
-      <c r="C110" s="102"/>
-    </row>
-    <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B111" s="101" t="s">
+    <row r="120" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B120" s="115"/>
+      <c r="C120" s="116"/>
+    </row>
+    <row r="121" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B121" s="115" t="s">
         <v>117</v>
       </c>
-      <c r="C111" s="102" t="s">
-        <v>318</v>
-      </c>
-      <c r="F111" s="6" t="n">
+      <c r="C121" s="116" t="s">
+        <v>367</v>
+      </c>
+      <c r="F121" s="6" t="n">
         <v>211</v>
       </c>
-      <c r="G111" s="7" t="s">
+      <c r="G121" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B112" s="101"/>
-      <c r="C112" s="102"/>
-    </row>
-    <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B113" s="101" t="s">
+    <row r="122" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B122" s="115"/>
+      <c r="C122" s="116"/>
+    </row>
+    <row r="123" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B123" s="115" t="s">
         <v>127</v>
       </c>
-      <c r="C113" s="102" t="s">
-        <v>319</v>
+      <c r="C123" s="116" t="s">
+        <v>368</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="37">
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="L3:M3"/>
     <mergeCell ref="N5:O5"/>
@@ -5943,6 +6738,24 @@
     <mergeCell ref="R79:V79"/>
     <mergeCell ref="K83:L83"/>
     <mergeCell ref="M83:N83"/>
+    <mergeCell ref="I89:J89"/>
+    <mergeCell ref="I90:J90"/>
+    <mergeCell ref="K90:L90"/>
+    <mergeCell ref="I91:J91"/>
+    <mergeCell ref="K91:L91"/>
+    <mergeCell ref="I92:J92"/>
+    <mergeCell ref="K92:L92"/>
+    <mergeCell ref="M93:N93"/>
+    <mergeCell ref="S93:T93"/>
+    <mergeCell ref="U93:V93"/>
+    <mergeCell ref="W93:X93"/>
+    <mergeCell ref="Y93:Z93"/>
+    <mergeCell ref="M94:N94"/>
+    <mergeCell ref="S94:T94"/>
+    <mergeCell ref="U94:V94"/>
+    <mergeCell ref="W94:X94"/>
+    <mergeCell ref="Y94:Z94"/>
+    <mergeCell ref="I95:J95"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.708333333333333" right="0.708333333333333" top="0.747916666666667" bottom="0.747916666666667" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Vaccum sensor and Pop truncade fix
</commit_message>
<xml_diff>
--- a/PGN 5.7_planter.xlsx
+++ b/PGN 5.7_planter.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="375">
   <si>
     <t xml:space="preserve">PGN Name</t>
   </si>
@@ -904,10 +904,19 @@
     <t xml:space="preserve">A2</t>
   </si>
   <si>
-    <t xml:space="preserve">inWC1X10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">inWC2X10</t>
+    <t xml:space="preserve">Raw1Left Hi/Lo 0-4095(0-12v)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw2Rgh Hi/Lo 0-4095(0-12v)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InWC1X10-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InWC2X10-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For 0 it send 5</t>
   </si>
   <si>
     <t xml:space="preserve">Vacuum config</t>
@@ -1913,18 +1922,22 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1935,10 +1948,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -5300,26 +5309,28 @@
         <v>8</v>
       </c>
       <c r="I91" s="100" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="J91" s="100"/>
       <c r="K91" s="100" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="L91" s="100"/>
       <c r="M91" s="8" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="N91" s="8" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="O91" s="8"/>
       <c r="P91" s="8"/>
       <c r="Q91" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="R91" s="8"/>
-      <c r="S91" s="8"/>
+      <c r="R91" s="87" t="s">
+        <v>297</v>
+      </c>
+      <c r="S91" s="87"/>
       <c r="T91" s="8"/>
       <c r="U91" s="8"/>
       <c r="V91" s="8"/>
@@ -5345,7 +5356,7 @@
     <row r="92" s="59" customFormat="true" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="49"/>
       <c r="C92" s="102" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D92" s="96" t="s">
         <v>102</v>
@@ -5354,7 +5365,7 @@
         <v>123</v>
       </c>
       <c r="F92" s="98" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="G92" s="99" t="n">
         <v>163</v>
@@ -5363,18 +5374,18 @@
         <v>8</v>
       </c>
       <c r="I92" s="103" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="J92" s="103"/>
       <c r="K92" s="103" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="L92" s="103"/>
       <c r="M92" s="103" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="N92" s="103" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="O92" s="100"/>
       <c r="P92" s="8"/>
@@ -5407,8 +5418,8 @@
     </row>
     <row r="93" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="49"/>
-      <c r="C93" s="102" t="s">
-        <v>300</v>
+      <c r="C93" s="105" t="s">
+        <v>303</v>
       </c>
       <c r="D93" s="96" t="s">
         <v>102</v>
@@ -5417,7 +5428,7 @@
         <v>123</v>
       </c>
       <c r="F93" s="98" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="G93" s="99" t="n">
         <v>164</v>
@@ -5426,13 +5437,13 @@
         <v>8</v>
       </c>
       <c r="I93" s="9" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J93" s="8" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="K93" s="8" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="L93" s="101"/>
       <c r="M93" s="100" t="s">
@@ -5440,31 +5451,31 @@
       </c>
       <c r="N93" s="100"/>
       <c r="O93" s="8" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="P93" s="8" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="Q93" s="87" t="s">
         <v>25</v>
       </c>
       <c r="R93" s="8" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="S93" s="87" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="T93" s="87"/>
       <c r="U93" s="8" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="V93" s="8"/>
       <c r="W93" s="8" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="X93" s="8"/>
       <c r="Y93" s="8" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="Z93" s="8"/>
       <c r="AA93" s="8"/>
@@ -5484,8 +5495,8 @@
     </row>
     <row r="94" s="59" customFormat="true" ht="30.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="49"/>
-      <c r="C94" s="105" t="s">
-        <v>312</v>
+      <c r="C94" s="106" t="s">
+        <v>315</v>
       </c>
       <c r="D94" s="96" t="s">
         <v>102</v>
@@ -5494,7 +5505,7 @@
         <v>123</v>
       </c>
       <c r="F94" s="98" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G94" s="99" t="n">
         <v>165</v>
@@ -5502,46 +5513,46 @@
       <c r="H94" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="I94" s="106" t="s">
-        <v>314</v>
-      </c>
-      <c r="J94" s="106" t="s">
-        <v>314</v>
-      </c>
-      <c r="K94" s="106" t="s">
-        <v>314</v>
-      </c>
-      <c r="L94" s="107" t="s">
-        <v>315</v>
-      </c>
-      <c r="M94" s="107" t="s">
+      <c r="I94" s="107" t="s">
+        <v>317</v>
+      </c>
+      <c r="J94" s="107" t="s">
+        <v>317</v>
+      </c>
+      <c r="K94" s="107" t="s">
+        <v>317</v>
+      </c>
+      <c r="L94" s="108" t="s">
+        <v>318</v>
+      </c>
+      <c r="M94" s="108" t="s">
         <v>287</v>
       </c>
-      <c r="N94" s="107"/>
+      <c r="N94" s="108"/>
       <c r="O94" s="103" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="P94" s="87" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="Q94" s="87" t="s">
         <v>25</v>
       </c>
       <c r="R94" s="87" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="S94" s="87" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="T94" s="87"/>
       <c r="U94" s="87" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="V94" s="87"/>
       <c r="W94" s="87"/>
       <c r="X94" s="87"/>
       <c r="Y94" s="87" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="Z94" s="87"/>
       <c r="AA94" s="8"/>
@@ -5561,8 +5572,8 @@
     </row>
     <row r="95" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="49"/>
-      <c r="C95" s="108" t="s">
-        <v>319</v>
+      <c r="C95" s="102" t="s">
+        <v>322</v>
       </c>
       <c r="D95" s="96" t="s">
         <v>102</v>
@@ -5571,7 +5582,7 @@
         <v>123</v>
       </c>
       <c r="F95" s="98" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G95" s="99" t="n">
         <v>166</v>
@@ -5580,20 +5591,20 @@
         <v>8</v>
       </c>
       <c r="I95" s="100" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="J95" s="100"/>
       <c r="K95" s="8" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="L95" s="8" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="M95" s="8" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="N95" s="8" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="O95" s="8"/>
       <c r="P95" s="8"/>
@@ -5601,7 +5612,7 @@
         <v>25</v>
       </c>
       <c r="R95" s="87" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="S95" s="87"/>
       <c r="T95" s="87"/>
@@ -5628,8 +5639,8 @@
     </row>
     <row r="96" s="59" customFormat="true" ht="27.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B96" s="49"/>
-      <c r="C96" s="108" t="s">
-        <v>327</v>
+      <c r="C96" s="102" t="s">
+        <v>330</v>
       </c>
       <c r="D96" s="96" t="s">
         <v>102</v>
@@ -5638,7 +5649,7 @@
         <v>123</v>
       </c>
       <c r="F96" s="98" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="G96" s="99" t="n">
         <v>167</v>
@@ -5647,18 +5658,18 @@
         <v>8</v>
       </c>
       <c r="I96" s="103" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="J96" s="103"/>
       <c r="K96" s="103" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="L96" s="103"/>
       <c r="M96" s="8" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="N96" s="8" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="O96" s="8"/>
       <c r="P96" s="8"/>
@@ -5773,10 +5784,10 @@
     </row>
     <row r="99" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="49" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>17</v>
@@ -5790,7 +5801,7 @@
         <v>3</v>
       </c>
       <c r="I99" s="9" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="J99" s="8" t="n">
         <v>0</v>
@@ -5873,10 +5884,10 @@
     </row>
     <row r="101" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="49" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D101" s="4" t="n">
         <v>126</v>
@@ -5890,19 +5901,19 @@
         <v>5</v>
       </c>
       <c r="I101" s="9" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="J101" s="8" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K101" s="8" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="L101" s="8" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="M101" s="8" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="N101" s="8" t="s">
         <v>25</v>
@@ -5937,7 +5948,7 @@
     <row r="102" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B102" s="109"/>
       <c r="C102" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D102" s="4" t="n">
         <v>123</v>
@@ -5951,10 +5962,10 @@
         <v>5</v>
       </c>
       <c r="I102" s="9" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J102" s="8" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="K102" s="8" t="s">
         <v>57</v>
@@ -5998,7 +6009,7 @@
     <row r="103" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B103" s="109"/>
       <c r="C103" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D103" s="4" t="n">
         <v>121</v>
@@ -6059,7 +6070,7 @@
     <row r="104" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B104" s="109"/>
       <c r="C104" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D104" s="4" t="n">
         <v>120</v>
@@ -6160,10 +6171,10 @@
     </row>
     <row r="106" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="49" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>17</v>
@@ -6183,13 +6194,13 @@
         <v>201</v>
       </c>
       <c r="K106" s="8" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="L106" s="8" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="M106" s="8" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="N106" s="8" t="s">
         <v>25</v>
@@ -6264,10 +6275,10 @@
     </row>
     <row r="108" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B108" s="49" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C108" s="110" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>17</v>
@@ -6364,10 +6375,10 @@
     </row>
     <row r="110" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B110" s="49" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="D110" s="111" t="n">
         <v>126</v>
@@ -6381,25 +6392,25 @@
         <v>7</v>
       </c>
       <c r="I110" s="9" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J110" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="K110" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="L110" s="8" t="n">
         <v>126</v>
       </c>
       <c r="M110" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="N110" s="8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="O110" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="P110" s="8" t="s">
         <v>25</v>
@@ -6432,7 +6443,7 @@
     <row r="111" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B111" s="49"/>
       <c r="C111" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D111" s="111" t="n">
         <v>123</v>
@@ -6446,25 +6457,25 @@
         <v>7</v>
       </c>
       <c r="I111" s="9" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J111" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="K111" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="L111" s="8" t="n">
         <v>123</v>
       </c>
       <c r="M111" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="N111" s="8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="O111" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="P111" s="8" t="s">
         <v>25</v>
@@ -6497,7 +6508,7 @@
     <row r="112" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B112" s="49"/>
       <c r="C112" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="D112" s="111" t="n">
         <v>121</v>
@@ -6511,25 +6522,25 @@
         <v>7</v>
       </c>
       <c r="I112" s="9" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J112" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="K112" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="L112" s="8" t="n">
         <v>121</v>
       </c>
       <c r="M112" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="N112" s="8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="O112" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="P112" s="8" t="s">
         <v>25</v>
@@ -6562,7 +6573,7 @@
     <row r="113" s="59" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="49"/>
       <c r="C113" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D113" s="111" t="n">
         <v>120</v>
@@ -6576,25 +6587,25 @@
         <v>7</v>
       </c>
       <c r="I113" s="9" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J113" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="K113" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="L113" s="8" t="n">
         <v>120</v>
       </c>
       <c r="M113" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="N113" s="8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="O113" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="P113" s="8" t="s">
         <v>25</v>
@@ -6667,14 +6678,14 @@
     </row>
     <row r="116" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C116" s="112" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D116" s="113" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E116" s="114"/>
       <c r="F116" s="115" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="G116" s="56"/>
     </row>
@@ -6683,7 +6694,7 @@
         <v>15</v>
       </c>
       <c r="C117" s="117" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D117" s="4" t="n">
         <v>254</v>
@@ -6707,7 +6718,7 @@
         <v>59</v>
       </c>
       <c r="C119" s="117" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="D119" s="4" t="n">
         <v>239</v>
@@ -6731,7 +6742,7 @@
         <v>117</v>
       </c>
       <c r="C121" s="117" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F121" s="6" t="n">
         <v>211</v>
@@ -6749,11 +6760,11 @@
         <v>127</v>
       </c>
       <c r="C123" s="117" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="41">
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="L3:M3"/>
     <mergeCell ref="N5:O5"/>
@@ -6778,6 +6789,7 @@
     <mergeCell ref="K90:L90"/>
     <mergeCell ref="I91:J91"/>
     <mergeCell ref="K91:L91"/>
+    <mergeCell ref="R91:S91"/>
     <mergeCell ref="I92:J92"/>
     <mergeCell ref="K92:L92"/>
     <mergeCell ref="M93:N93"/>

</xml_diff>